<commit_message>
Lo que se hizo hoy
</commit_message>
<xml_diff>
--- a/documentos/Cronograma_semanal Proyecto .xlsx
+++ b/documentos/Cronograma_semanal Proyecto .xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SENA\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{95EE0A0B-5EF1-4AD9-BA1F-25AD26B937E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4213291-C19D-4734-8FFA-AF5A19B105A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="1470" windowWidth="15615" windowHeight="14730" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cronograma semanal" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t>CRONOGRAMA SEMANAL DE ACTIVIDADES</t>
   </si>
@@ -157,6 +157,12 @@
   </si>
   <si>
     <t>Se agregó un nuevo apartado de opiniones en el cual los clientes dan opiniones sobre los abogados</t>
+  </si>
+  <si>
+    <t>se mejoró el diseño de las interfaces nosostros, servicios y contactos</t>
+  </si>
+  <si>
+    <t>se arreglaron erros en algunos apartados y se agregaron nuevos botones</t>
   </si>
 </sst>
 </file>
@@ -817,7 +823,9 @@
       <c r="E10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="9"/>
+      <c r="F10" s="9" t="s">
+        <v>32</v>
+      </c>
       <c r="G10" s="9"/>
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
@@ -838,7 +846,9 @@
       <c r="E11" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="9"/>
+      <c r="F11" s="9" t="s">
+        <v>33</v>
+      </c>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
@@ -856,8 +866,12 @@
       <c r="D12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
+      <c r="E12" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>29</v>
+      </c>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
       <c r="I12" s="9"/>

</xml_diff>